<commit_message>
Cập nhật tài liệu QA 018, xoá QA 012 và cập nhật backlog export
- docs/QA/018: rà soát lại fail-fast khi thiếu secret (2026-09-27) cho cả
  orders và baskets; ghi rõ baseline `${VAR:-default}` của Compose và bẫy
  đặt biến `.env` thành chuỗi rỗng
- docs/QA/QA_Debt.md: thêm mục rà soát lại 018 (2026-09-27)
- Xoá docs/QA/012_QA_cổng chất lượng SonarQube.md
- Cập nhật docs/requirement/SCRUM_Backlog_Export.xlsx

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirement/SCRUM_Backlog_Export.xlsx
+++ b/docs/requirement/SCRUM_Backlog_Export.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngantran\source\repos\ecomerce\docs\requirement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E8CCF02-BBD1-4A6C-9AE1-B3BD770CC61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300"/>
   </bookViews>
   <sheets>
     <sheet name="SCRUM Tickets" sheetId="1" r:id="rId1"/>
@@ -1055,7 +1054,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1409,7 +1408,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2647,7 +2646,7 @@
         <v>54</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>23</v>
@@ -2735,7 +2734,7 @@
         <v>54</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>23</v>
@@ -2989,7 +2988,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N37" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:N37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>